<commit_message>
Update done and new  artifacts added...
</commit_message>
<xml_diff>
--- a/Reports/txpa_corr_factors_be_cold_estimates.xlsx
+++ b/Reports/txpa_corr_factors_be_cold_estimates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UserData\Learning\Software_Programming\GitHub_Nelio92\Tasks_Automation_Code\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11E0B95-B26E-4CB2-BF62-D3B03741C583}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7824D5AE-7C5C-48D0-B759-BA14E7E08434}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22240" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -807,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y64"/>
+  <dimension ref="A1:Z64"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -817,19 +817,18 @@
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="4" customWidth="1"/>
-    <col min="8" max="11" width="23" customWidth="1"/>
-    <col min="12" max="12" width="23" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="12" width="23" customWidth="1"/>
     <col min="13" max="13" width="22" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="14" max="14" width="23" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="15" max="15" width="22" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="16" max="17" width="23" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="18" max="18" width="23" customWidth="1" collapsed="1"/>
-    <col min="19" max="19" width="29" customWidth="1"/>
-    <col min="20" max="20" width="24" customWidth="1"/>
-    <col min="21" max="21" width="23" customWidth="1"/>
-    <col min="22" max="22" width="26" customWidth="1"/>
+    <col min="16" max="18" width="23" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="19" max="19" width="29" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="20" max="20" width="24" customWidth="1" collapsed="1"/>
+    <col min="21" max="21" width="23" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="22" width="26" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="23" max="24" width="40" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="25" width="28" customWidth="1" collapsed="1"/>
+    <col min="25" max="25" width="28" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="8.7265625" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -866,7 +865,7 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="11" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
@@ -893,7 +892,7 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="V1" s="1" t="s">
@@ -943,7 +942,7 @@
       <c r="K2" s="3">
         <v>2.0000313499999982</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="12">
         <v>-0.34888240809258098</v>
       </c>
       <c r="M2" s="3">
@@ -970,7 +969,7 @@
       <c r="T2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="12">
+      <c r="U2" s="3">
         <v>-0.73321614570023286</v>
       </c>
       <c r="V2" s="3" t="s">
@@ -1020,7 +1019,7 @@
       <c r="K3" s="6">
         <v>4.4187675000000093E-2</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="13">
         <v>1.073758704862003</v>
       </c>
       <c r="M3" s="6">
@@ -1047,7 +1046,7 @@
       <c r="T3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U3" s="13">
+      <c r="U3" s="6">
         <v>1.0998696037256399</v>
       </c>
       <c r="V3" s="6" t="s">
@@ -1097,7 +1096,7 @@
       <c r="K4" s="6">
         <v>1.9182050000000169E-2</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="13">
         <v>0.92119049099836703</v>
       </c>
       <c r="M4" s="6">
@@ -1124,7 +1123,7 @@
       <c r="T4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U4" s="13">
+      <c r="U4" s="6">
         <v>0.93252533872563981</v>
       </c>
       <c r="V4" s="6" t="s">
@@ -1174,7 +1173,7 @@
       <c r="K5" s="6">
         <v>8.2940569349999937E-2</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="13">
         <v>0.83441548594154913</v>
       </c>
       <c r="M5" s="6">
@@ -1201,7 +1200,7 @@
       <c r="T5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U5" s="13">
+      <c r="U5" s="6">
         <v>0.81847730626371928</v>
       </c>
       <c r="V5" s="6" t="s">
@@ -1251,7 +1250,7 @@
       <c r="K6" s="6">
         <v>0.15286255000000001</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="13">
         <v>0.77854956327109448</v>
       </c>
       <c r="M6" s="6">
@@ -1278,7 +1277,7 @@
       <c r="T6" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U6" s="13">
+      <c r="U6" s="6">
         <v>0.74917490612797644</v>
       </c>
       <c r="V6" s="6" t="s">
@@ -1328,7 +1327,7 @@
       <c r="K7" s="6">
         <v>0.14885554999999989</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="13">
         <v>0.83786888599836751</v>
       </c>
       <c r="M7" s="6">
@@ -1355,7 +1354,7 @@
       <c r="T7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U7" s="13">
+      <c r="U7" s="6">
         <v>0.80926422942878729</v>
       </c>
       <c r="V7" s="6" t="s">
@@ -1405,7 +1404,7 @@
       <c r="K8" s="6">
         <v>0.1161737350000009</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="13">
         <v>0.9773786725892758</v>
       </c>
       <c r="M8" s="6">
@@ -1432,7 +1431,7 @@
       <c r="T8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U8" s="13">
+      <c r="U8" s="6">
         <v>0.95505427963193967</v>
       </c>
       <c r="V8" s="6" t="s">
@@ -1482,7 +1481,7 @@
       <c r="K9" s="6">
         <v>0.10741802500004009</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="13">
         <v>1.051847086225576</v>
       </c>
       <c r="M9" s="6">
@@ -1509,7 +1508,7 @@
       <c r="T9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U9" s="13">
+      <c r="U9" s="6">
         <v>1.031205224269413</v>
       </c>
       <c r="V9" s="6" t="s">
@@ -1559,7 +1558,7 @@
       <c r="K10" s="6">
         <v>7.653728000000104E-2</v>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="13">
         <v>1.151378259180144</v>
       </c>
       <c r="M10" s="6">
@@ -1586,7 +1585,7 @@
       <c r="T10" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U10" s="13">
+      <c r="U10" s="6">
         <v>1.136670560278962</v>
       </c>
       <c r="V10" s="6" t="s">
@@ -1636,7 +1635,7 @@
       <c r="K11" s="6">
         <v>4.3889429999999008E-2</v>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="13">
         <v>1.257917785543782</v>
       </c>
       <c r="M11" s="6">
@@ -1663,7 +1662,7 @@
       <c r="T11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U11" s="13">
+      <c r="U11" s="6">
         <v>1.2838524487256</v>
       </c>
       <c r="V11" s="6" t="s">
@@ -1713,7 +1712,7 @@
       <c r="K12" s="6">
         <v>3.4861805000000023E-2</v>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="13">
         <v>1.2992827912256</v>
       </c>
       <c r="M12" s="6">
@@ -1740,7 +1739,7 @@
       <c r="T12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U12" s="13">
+      <c r="U12" s="6">
         <v>1.3198829487256001</v>
       </c>
       <c r="V12" s="6" t="s">
@@ -1790,7 +1789,7 @@
       <c r="K13" s="6">
         <v>1.961354999999898E-2</v>
       </c>
-      <c r="L13" s="6">
+      <c r="L13" s="13">
         <v>1.3931537237256</v>
       </c>
       <c r="M13" s="6">
@@ -1817,7 +1816,7 @@
       <c r="T13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U13" s="13">
+      <c r="U13" s="6">
         <v>1.3815638987256</v>
       </c>
       <c r="V13" s="6" t="s">
@@ -1867,7 +1866,7 @@
       <c r="K14" s="6">
         <v>0.15665330000000099</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="13">
         <v>1.6362978078165109</v>
       </c>
       <c r="M14" s="6">
@@ -1894,7 +1893,7 @@
       <c r="T14" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U14" s="13">
+      <c r="U14" s="6">
         <v>1.666400910099169</v>
       </c>
       <c r="V14" s="6" t="s">
@@ -1944,7 +1943,7 @@
       <c r="K15" s="6">
         <v>0.24602280000000001</v>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="13">
         <v>1.8646155078165081</v>
       </c>
       <c r="M15" s="6">
@@ -1971,7 +1970,7 @@
       <c r="T15" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U15" s="13">
+      <c r="U15" s="6">
         <v>1.9118921978847421</v>
       </c>
       <c r="V15" s="6" t="s">
@@ -2021,7 +2020,7 @@
       <c r="K16" s="6">
         <v>0.34880250000000212</v>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="13">
         <v>1.77500286690742</v>
       </c>
       <c r="M16" s="6">
@@ -2048,7 +2047,7 @@
       <c r="T16" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U16" s="13">
+      <c r="U16" s="6">
         <v>1.842030100511481</v>
       </c>
       <c r="V16" s="6" t="s">
@@ -2098,7 +2097,7 @@
       <c r="K17" s="6">
         <v>4.3629600000001163E-2</v>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="13">
         <v>1.317227771452872</v>
       </c>
       <c r="M17" s="6">
@@ -2125,7 +2124,7 @@
       <c r="T17" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U17" s="13">
+      <c r="U17" s="6">
         <v>1.3430088987255999</v>
       </c>
       <c r="V17" s="6" t="s">
@@ -2175,7 +2174,7 @@
       <c r="K18" s="6">
         <v>0.28397700000000009</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="13">
         <v>1.6444986896346909</v>
       </c>
       <c r="M18" s="6">
@@ -2202,7 +2201,7 @@
       <c r="T18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U18" s="13">
+      <c r="U18" s="6">
         <v>1.6990688051504359</v>
       </c>
       <c r="V18" s="6" t="s">
@@ -2252,7 +2251,7 @@
       <c r="K19" s="6">
         <v>3.409470000000181E-2</v>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="13">
         <v>1.36301406690742</v>
       </c>
       <c r="M19" s="6">
@@ -2279,7 +2278,7 @@
       <c r="T19" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U19" s="13">
+      <c r="U19" s="6">
         <v>1.3428671987256009</v>
       </c>
       <c r="V19" s="6" t="s">
@@ -2329,7 +2328,7 @@
       <c r="K20" s="6">
         <v>0.22494829999999899</v>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="13">
         <v>1.737982794180144</v>
       </c>
       <c r="M20" s="6">
@@ -2356,7 +2355,7 @@
       <c r="T20" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U20" s="13">
+      <c r="U20" s="6">
         <v>1.7812097270517151</v>
       </c>
       <c r="V20" s="6" t="s">
@@ -2406,7 +2405,7 @@
       <c r="K21" s="6">
         <v>7.8146500000001895E-2</v>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="13">
         <v>1.4224194214528709</v>
       </c>
       <c r="M21" s="6">
@@ -2433,7 +2432,7 @@
       <c r="T21" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U21" s="13">
+      <c r="U21" s="6">
         <v>1.407402488630314</v>
       </c>
       <c r="V21" s="6" t="s">
@@ -2483,7 +2482,7 @@
       <c r="K22" s="9">
         <v>0.165934</v>
       </c>
-      <c r="L22" s="9">
+      <c r="L22" s="14">
         <v>1.9138830078165081</v>
       </c>
       <c r="M22" s="9">
@@ -2510,7 +2509,7 @@
       <c r="T22" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="U22" s="14">
+      <c r="U22" s="9">
         <v>1.9457695252034419</v>
       </c>
       <c r="V22" s="9" t="s">
@@ -2560,7 +2559,7 @@
       <c r="K23" s="3">
         <v>2.2030029</v>
       </c>
-      <c r="L23" s="3">
+      <c r="L23" s="12">
         <v>-0.76873509958178987</v>
       </c>
       <c r="M23" s="3">
@@ -2587,7 +2586,7 @@
       <c r="T23" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="U23" s="12">
+      <c r="U23" s="3">
         <v>-1.192072633024708</v>
       </c>
       <c r="V23" s="3" t="s">
@@ -2637,7 +2636,7 @@
       <c r="K24" s="6">
         <v>0.1770106650000054</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="13">
         <v>1.0732586874636321</v>
       </c>
       <c r="M24" s="6">
@@ -2664,7 +2663,7 @@
       <c r="T24" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U24" s="13">
+      <c r="U24" s="6">
         <v>1.1072737395156249</v>
       </c>
       <c r="V24" s="6" t="s">
@@ -2714,7 +2713,7 @@
       <c r="K25" s="6">
         <v>0.19283388500000001</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="13">
         <v>0.91754823200908819</v>
       </c>
       <c r="M25" s="6">
@@ -2741,7 +2740,7 @@
       <c r="T25" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U25" s="13">
+      <c r="U25" s="6">
         <v>0.95460393504067076</v>
       </c>
       <c r="V25" s="6" t="s">
@@ -2791,7 +2790,7 @@
       <c r="K26" s="6">
         <v>9.9990486999998129E-2</v>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="13">
         <v>0.7745990380999942</v>
       </c>
       <c r="M26" s="6">
@@ -2818,7 +2817,7 @@
       <c r="T26" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U26" s="13">
+      <c r="U26" s="6">
         <v>0.79381359570876331</v>
       </c>
       <c r="V26" s="6" t="s">
@@ -2868,7 +2867,7 @@
       <c r="K27" s="6">
         <v>2.7679669999999931E-2</v>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="13">
         <v>0.7031988849636337</v>
       </c>
       <c r="M27" s="6">
@@ -2895,7 +2894,7 @@
       <c r="T27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U27" s="13">
+      <c r="U27" s="6">
         <v>0.68684271632727012</v>
       </c>
       <c r="V27" s="6" t="s">
@@ -2945,7 +2944,7 @@
       <c r="K28" s="6">
         <v>6.8182999999999439E-4</v>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="13">
         <v>0.70200038678181564</v>
       </c>
       <c r="M28" s="6">
@@ -2972,7 +2971,7 @@
       <c r="T28" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U28" s="13">
+      <c r="U28" s="6">
         <v>0.70240328632727023</v>
       </c>
       <c r="V28" s="6" t="s">
@@ -3022,7 +3021,7 @@
       <c r="K29" s="6">
         <v>4.2718535000000113E-2</v>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="13">
         <v>0.70829444064545133</v>
       </c>
       <c r="M29" s="6">
@@ -3049,7 +3048,7 @@
       <c r="T29" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U29" s="13">
+      <c r="U29" s="6">
         <v>0.73353721132726957</v>
       </c>
       <c r="V29" s="6" t="s">
@@ -3099,7 +3098,7 @@
       <c r="K30" s="6">
         <v>5.773226999999892E-2</v>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="13">
         <v>0.73742498814545343</v>
       </c>
       <c r="M30" s="6">
@@ -3126,7 +3125,7 @@
       <c r="T30" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U30" s="13">
+      <c r="U30" s="6">
         <v>0.72633093248993874</v>
       </c>
       <c r="V30" s="6" t="s">
@@ -3176,7 +3175,7 @@
       <c r="K31" s="6">
         <v>5.560860000000023E-2</v>
       </c>
-      <c r="L31" s="6">
+      <c r="L31" s="13">
         <v>0.80045791905457253</v>
       </c>
       <c r="M31" s="6">
@@ -3203,7 +3202,7 @@
       <c r="T31" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U31" s="13">
+      <c r="U31" s="6">
         <v>0.78977195601647843</v>
       </c>
       <c r="V31" s="6" t="s">
@@ -3253,7 +3252,7 @@
       <c r="K32" s="6">
         <v>6.5547949999995581E-3</v>
       </c>
-      <c r="L32" s="6">
+      <c r="L32" s="13">
         <v>0.9108849533727551</v>
       </c>
       <c r="M32" s="6">
@@ -3280,7 +3279,7 @@
       <c r="T32" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U32" s="13">
+      <c r="U32" s="6">
         <v>0.91475824132730033</v>
       </c>
       <c r="V32" s="6" t="s">
@@ -3330,7 +3329,7 @@
       <c r="K33" s="6">
         <v>2.1854569999999459E-2</v>
       </c>
-      <c r="L33" s="6">
+      <c r="L33" s="13">
         <v>0.96196085541820853</v>
       </c>
       <c r="M33" s="6">
@@ -3357,7 +3356,7 @@
       <c r="T33" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U33" s="13">
+      <c r="U33" s="6">
         <v>0.94904679132729974</v>
       </c>
       <c r="V33" s="6" t="s">
@@ -3407,7 +3406,7 @@
       <c r="K34" s="6">
         <v>2.3850549999998801E-2</v>
       </c>
-      <c r="L34" s="6">
+      <c r="L34" s="13">
         <v>0.98753739814548069</v>
       </c>
       <c r="M34" s="6">
@@ -3434,7 +3433,7 @@
       <c r="T34" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U34" s="13">
+      <c r="U34" s="6">
         <v>0.97344389132729958</v>
       </c>
       <c r="V34" s="6" t="s">
@@ -3484,7 +3483,7 @@
       <c r="K35" s="6">
         <v>0.21216860000000029</v>
       </c>
-      <c r="L35" s="6">
+      <c r="L35" s="13">
         <v>1.227122095872756</v>
       </c>
       <c r="M35" s="6">
@@ -3511,7 +3510,7 @@
       <c r="T35" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U35" s="13">
+      <c r="U35" s="6">
         <v>1.267893232305684</v>
       </c>
       <c r="V35" s="6" t="s">
@@ -3561,7 +3560,7 @@
       <c r="K36" s="6">
         <v>0.13043380000000049</v>
       </c>
-      <c r="L36" s="6">
+      <c r="L36" s="13">
         <v>0.84754895950911857</v>
       </c>
       <c r="M36" s="6">
@@ -3588,7 +3587,7 @@
       <c r="T36" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U36" s="13">
+      <c r="U36" s="6">
         <v>0.87261362155272604</v>
       </c>
       <c r="V36" s="6" t="s">
@@ -3638,7 +3637,7 @@
       <c r="K37" s="6">
         <v>0.37290139999999861</v>
       </c>
-      <c r="L37" s="6">
+      <c r="L37" s="13">
         <v>1.330331368600026</v>
       </c>
       <c r="M37" s="6">
@@ -3665,7 +3664,7 @@
       <c r="T37" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U37" s="13">
+      <c r="U37" s="6">
         <v>1.4019895397687581</v>
       </c>
       <c r="V37" s="6" t="s">
@@ -3715,7 +3714,7 @@
       <c r="K38" s="6">
         <v>0.32259959999999999</v>
       </c>
-      <c r="L38" s="6">
+      <c r="L38" s="13">
         <v>1.615507177690936</v>
       </c>
       <c r="M38" s="6">
@@ -3742,7 +3741,7 @@
       <c r="T38" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U38" s="13">
+      <c r="U38" s="6">
         <v>1.677499160975966</v>
       </c>
       <c r="V38" s="6" t="s">
@@ -3792,7 +3791,7 @@
       <c r="K39" s="6">
         <v>0.33581929999999921</v>
       </c>
-      <c r="L39" s="6">
+      <c r="L39" s="13">
         <v>1.307447618600027</v>
       </c>
       <c r="M39" s="6">
@@ -3819,7 +3818,7 @@
       <c r="T39" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U39" s="13">
+      <c r="U39" s="6">
         <v>1.371979950420618</v>
       </c>
       <c r="V39" s="6" t="s">
@@ -3869,7 +3868,7 @@
       <c r="K40" s="6">
         <v>0.38128420000000102</v>
       </c>
-      <c r="L40" s="6">
+      <c r="L40" s="13">
         <v>1.8334782413273021</v>
       </c>
       <c r="M40" s="6">
@@ -3896,7 +3895,7 @@
       <c r="T40" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U40" s="13">
+      <c r="U40" s="6">
         <v>1.9067472836734349</v>
       </c>
       <c r="V40" s="6" t="s">
@@ -3946,7 +3945,7 @@
       <c r="K41" s="6">
         <v>0.41202169999999788</v>
       </c>
-      <c r="L41" s="6">
+      <c r="L41" s="13">
         <v>1.7465384095091161</v>
       </c>
       <c r="M41" s="6">
@@ -3973,7 +3972,7 @@
       <c r="T41" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U41" s="13">
+      <c r="U41" s="6">
         <v>1.825714088398579</v>
       </c>
       <c r="V41" s="6" t="s">
@@ -4023,7 +4022,7 @@
       <c r="K42" s="6">
         <v>0.19407510000000089</v>
       </c>
-      <c r="L42" s="6">
+      <c r="L42" s="13">
         <v>1.601665982236391</v>
       </c>
       <c r="M42" s="6">
@@ -4050,7 +4049,7 @@
       <c r="T42" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U42" s="13">
+      <c r="U42" s="6">
         <v>1.6389602019292879</v>
       </c>
       <c r="V42" s="6" t="s">
@@ -4100,7 +4099,7 @@
       <c r="K43" s="9">
         <v>9.1844999999999288E-2</v>
       </c>
-      <c r="L43" s="9">
+      <c r="L43" s="14">
         <v>0.9680125867818451</v>
       </c>
       <c r="M43" s="9">
@@ -4127,7 +4126,7 @@
       <c r="T43" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="U43" s="14">
+      <c r="U43" s="9">
         <v>0.98566187619452128</v>
       </c>
       <c r="V43" s="9" t="s">
@@ -4177,7 +4176,7 @@
       <c r="K44" s="3">
         <v>2.282422200000001</v>
       </c>
-      <c r="L44" s="3">
+      <c r="L44" s="12">
         <v>-1.4468922529385291</v>
       </c>
       <c r="M44" s="3">
@@ -4204,7 +4203,7 @@
       <c r="T44" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="U44" s="12">
+      <c r="U44" s="3">
         <v>-1.885491305360731</v>
       </c>
       <c r="V44" s="3" t="s">
@@ -4254,7 +4253,7 @@
       <c r="K45" s="6">
         <v>2.1541419999999201E-2</v>
       </c>
-      <c r="L45" s="6">
+      <c r="L45" s="13">
         <v>0.21179265524323981</v>
       </c>
       <c r="M45" s="6">
@@ -4281,7 +4280,7 @@
       <c r="T45" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U45" s="13">
+      <c r="U45" s="6">
         <v>0.19906363433414939</v>
       </c>
       <c r="V45" s="6" t="s">
@@ -4331,7 +4330,7 @@
       <c r="K46" s="6">
         <v>5.7866739999999812E-2</v>
       </c>
-      <c r="L46" s="6">
+      <c r="L46" s="13">
         <v>2.568365706142264E-2</v>
       </c>
       <c r="M46" s="6">
@@ -4358,7 +4357,7 @@
       <c r="T46" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U46" s="13">
+      <c r="U46" s="6">
         <v>3.6803552990739341E-2</v>
       </c>
       <c r="V46" s="6" t="s">
@@ -4408,7 +4407,7 @@
       <c r="K47" s="6">
         <v>2.8277607999999881E-2</v>
       </c>
-      <c r="L47" s="6">
+      <c r="L47" s="13">
         <v>-0.15551947130221061</v>
       </c>
       <c r="M47" s="6">
@@ -4435,7 +4434,7 @@
       <c r="T47" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U47" s="13">
+      <c r="U47" s="6">
         <v>-0.13880997566584699</v>
       </c>
       <c r="V47" s="6" t="s">
@@ -4485,7 +4484,7 @@
       <c r="K48" s="6">
         <v>0.12682408000000001</v>
       </c>
-      <c r="L48" s="6">
+      <c r="L48" s="13">
         <v>-0.30708716248403212</v>
       </c>
       <c r="M48" s="6">
@@ -4512,7 +4511,7 @@
       <c r="T48" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U48" s="13">
+      <c r="U48" s="6">
         <v>-0.33145816681106588</v>
       </c>
       <c r="V48" s="6" t="s">
@@ -4562,7 +4561,7 @@
       <c r="K49" s="6">
         <v>0.15336623999999999</v>
       </c>
-      <c r="L49" s="6">
+      <c r="L49" s="13">
         <v>-0.31433587112039518</v>
       </c>
       <c r="M49" s="6">
@@ -4589,7 +4588,7 @@
       <c r="T49" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U49" s="13">
+      <c r="U49" s="6">
         <v>-0.34380731927646169</v>
       </c>
       <c r="V49" s="6" t="s">
@@ -4639,7 +4638,7 @@
       <c r="K50" s="6">
         <v>0.1361467549999999</v>
       </c>
-      <c r="L50" s="6">
+      <c r="L50" s="13">
         <v>-0.25240669589312298</v>
       </c>
       <c r="M50" s="6">
@@ -4666,7 +4665,7 @@
       <c r="T50" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U50" s="13">
+      <c r="U50" s="6">
         <v>-0.27856918140231463</v>
       </c>
       <c r="V50" s="6" t="s">
@@ -4716,7 +4715,7 @@
       <c r="K51" s="6">
         <v>0.112576035</v>
       </c>
-      <c r="L51" s="6">
+      <c r="L51" s="13">
         <v>-0.19298424816584969</v>
       </c>
       <c r="M51" s="6">
@@ -4743,7 +4742,7 @@
       <c r="T51" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U51" s="13">
+      <c r="U51" s="6">
         <v>-0.21461729321616899</v>
       </c>
       <c r="V51" s="6" t="s">
@@ -4793,7 +4792,7 @@
       <c r="K52" s="6">
         <v>8.1578529999950966E-2</v>
       </c>
-      <c r="L52" s="6">
+      <c r="L52" s="13">
         <v>-0.1223185056657714</v>
       </c>
       <c r="M52" s="6">
@@ -4820,7 +4819,7 @@
       <c r="T52" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U52" s="13">
+      <c r="U52" s="6">
         <v>-0.13799495060920661</v>
       </c>
       <c r="V52" s="6" t="s">
@@ -4870,7 +4869,7 @@
       <c r="K53" s="6">
         <v>6.0395485000000797E-2</v>
       </c>
-      <c r="L53" s="6">
+      <c r="L53" s="13">
         <v>-5.105314680216419E-2</v>
       </c>
       <c r="M53" s="6">
@@ -4897,7 +4896,7 @@
       <c r="T53" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U53" s="13">
+      <c r="U53" s="6">
         <v>-6.2658976123128429E-2</v>
       </c>
       <c r="V53" s="6" t="s">
@@ -4947,7 +4946,7 @@
       <c r="K54" s="6">
         <v>5.7267819999999858E-2</v>
       </c>
-      <c r="L54" s="6">
+      <c r="L54" s="13">
         <v>-2.222873112034485E-2</v>
       </c>
       <c r="M54" s="6">
@@ -4974,7 +4973,7 @@
       <c r="T54" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U54" s="13">
+      <c r="U54" s="6">
         <v>-3.3233536272645248E-2</v>
       </c>
       <c r="V54" s="6" t="s">
@@ -5024,7 +5023,7 @@
       <c r="K55" s="6">
         <v>6.5652309999999048E-2</v>
       </c>
-      <c r="L55" s="6">
+      <c r="L55" s="13">
         <v>-8.8635224839804481E-3</v>
       </c>
       <c r="M55" s="6">
@@ -5051,7 +5050,7 @@
       <c r="T55" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U55" s="13">
+      <c r="U55" s="6">
         <v>-2.1479523570601341E-2</v>
       </c>
       <c r="V55" s="6" t="s">
@@ -5101,7 +5100,7 @@
       <c r="K56" s="6">
         <v>7.0507499999999668E-2</v>
       </c>
-      <c r="L56" s="6">
+      <c r="L56" s="13">
         <v>0.18893654706147309</v>
       </c>
       <c r="M56" s="6">
@@ -5128,7 +5127,7 @@
       <c r="T56" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U56" s="13">
+      <c r="U56" s="6">
         <v>0.20248554018319201</v>
       </c>
       <c r="V56" s="6" t="s">
@@ -5178,7 +5177,7 @@
       <c r="K57" s="6">
         <v>0.16412209999999841</v>
       </c>
-      <c r="L57" s="6">
+      <c r="L57" s="13">
         <v>0.55280136524328904</v>
       </c>
       <c r="M57" s="6">
@@ -5205,7 +5204,7 @@
       <c r="T57" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U57" s="13">
+      <c r="U57" s="6">
         <v>0.5843397009383855</v>
       </c>
       <c r="V57" s="6" t="s">
@@ -5255,7 +5254,7 @@
       <c r="K58" s="6">
         <v>0.25847160000000008</v>
       </c>
-      <c r="L58" s="6">
+      <c r="L58" s="13">
         <v>0.38487154251601768</v>
       </c>
       <c r="M58" s="6">
@@ -5282,7 +5281,7 @@
       <c r="T58" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U58" s="13">
+      <c r="U58" s="6">
         <v>0.43454044200273412</v>
       </c>
       <c r="V58" s="6" t="s">
@@ -5332,7 +5331,7 @@
       <c r="K59" s="6">
         <v>3.1715000000005489E-3</v>
       </c>
-      <c r="L59" s="6">
+      <c r="L59" s="13">
         <v>7.5614856152380672E-2</v>
       </c>
       <c r="M59" s="6">
@@ -5359,7 +5358,7 @@
       <c r="T59" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U59" s="13">
+      <c r="U59" s="6">
         <v>7.7488924334199183E-2</v>
       </c>
       <c r="V59" s="6" t="s">
@@ -5409,7 +5408,7 @@
       <c r="K60" s="6">
         <v>0.2361500000000003</v>
       </c>
-      <c r="L60" s="6">
+      <c r="L60" s="13">
         <v>-5.4738293847618219E-2</v>
       </c>
       <c r="M60" s="6">
@@ -5436,7 +5435,7 @@
       <c r="T60" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="U60" s="13">
+      <c r="U60" s="6">
         <v>-9.3587991031744977E-3</v>
       </c>
       <c r="V60" s="6" t="s">
@@ -5486,7 +5485,7 @@
       <c r="K61" s="6">
         <v>7.404050000000062E-2</v>
       </c>
-      <c r="L61" s="6">
+      <c r="L61" s="13">
         <v>5.4596419788744063E-2</v>
       </c>
       <c r="M61" s="6">
@@ -5513,7 +5512,7 @@
       <c r="T61" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U61" s="13">
+      <c r="U61" s="6">
         <v>4.0368511761532222E-2</v>
       </c>
       <c r="V61" s="6" t="s">
@@ -5563,7 +5562,7 @@
       <c r="K62" s="6">
         <v>3.9973899999999681E-2</v>
       </c>
-      <c r="L62" s="6">
+      <c r="L62" s="13">
         <v>-7.1095916574890672E-2</v>
       </c>
       <c r="M62" s="6">
@@ -5590,7 +5589,7 @@
       <c r="T62" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="U62" s="13">
+      <c r="U62" s="6">
         <v>-4.7474975665799952E-2</v>
       </c>
       <c r="V62" s="6" t="s">
@@ -5640,7 +5639,7 @@
       <c r="K63" s="6">
         <v>0.1364184999999995</v>
       </c>
-      <c r="L63" s="6">
+      <c r="L63" s="13">
         <v>-2.1955007483981329E-2</v>
       </c>
       <c r="M63" s="6">
@@ -5667,7 +5666,7 @@
       <c r="T63" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U63" s="13">
+      <c r="U63" s="6">
         <v>-4.8169712560394373E-2</v>
       </c>
       <c r="V63" s="6" t="s">
@@ -5717,7 +5716,7 @@
       <c r="K64" s="9">
         <v>0.2060276999999999</v>
       </c>
-      <c r="L64" s="9">
+      <c r="L64" s="14">
         <v>0.42229346524329009</v>
       </c>
       <c r="M64" s="9">
@@ -5744,7 +5743,7 @@
       <c r="T64" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="U64" s="14">
+      <c r="U64" s="9">
         <v>0.46188454264900608</v>
       </c>
       <c r="V64" s="9" t="s">

</xml_diff>